<commit_message>
Design: style the Undergraduate page's new block variants
- cards (stats): navy / cyan / maize stat tiles with italic Aleo figures,
  tile colour authored per card via the card-style cell
- hero image-left + theme-light: maize portrait band, navy full-width CTA
- hero image-background-text-right + theme-dark: split navy CTA band,
  copy on the right half, cyan CTA
- cards.js: read card/CTA style from bare-text cells (DA) as well as <p>
- clear the fixed header on pages that open with a page title
- in-copy links (default content, columns): Roboto dotted underline,
  no floated chevron
- load Aleo 800/900 used by LSA headings and stat figures

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-audience-landing.report.xlsx
+++ b/tools/importer/reports/import-audience-landing.report.xlsx
@@ -64,7 +64,7 @@
     <t>department-landing</t>
   </si>
   <si>
-    <t>2026-10-07T15:51:15.956Z</t>
+    <t>2026-10-07T15:55:46.036Z</t>
   </si>
   <si>
     <t>Center for Global and Intercultural Study | U-M LSA</t>
@@ -148,7 +148,7 @@
     <t>unit-home</t>
   </si>
   <si>
-    <t>2026-10-07T15:51:04.207Z</t>
+    <t>2026-10-07T15:55:32.849Z</t>
   </si>
   <si>
     <t>Residential College | U-M LSA</t>
@@ -190,7 +190,7 @@
     <t>english/undergraduate</t>
   </si>
   <si>
-    <t>2026-10-07T15:51:08.681Z</t>
+    <t>2026-10-07T15:55:39.133Z</t>
   </si>
   <si>
     <t>Undergraduate Students | U-M LSA English Language and Literature</t>
@@ -211,7 +211,7 @@
     <t>about</t>
   </si>
   <si>
-    <t>2026-10-07T15:50:52.238Z</t>
+    <t>2026-10-07T15:55:26.327Z</t>
   </si>
   <si>
     <t>About | U-M LSA U-M College of LSA</t>
@@ -232,7 +232,7 @@
     <t>audience-landing</t>
   </si>
   <si>
-    <t>2026-10-07T15:55:17.283Z</t>
+    <t>2026-10-07T16:28:39.597Z</t>
   </si>
   <si>
     <t>Prospective Students | U-M LSA U-M College of LSA</t>
@@ -247,7 +247,7 @@
     <t>urop/prospective-students</t>
   </si>
   <si>
-    <t>2026-10-07T15:51:10.836Z</t>
+    <t>2026-10-07T15:55:42.084Z</t>
   </si>
   <si>
     <t>Prospective UROP Students | U-M LSA UROP: A Center for Research, Scholarship, and Creative Inquiry</t>
@@ -323,7 +323,7 @@
     <t>lsa/prospective-students/undergraduate</t>
   </si>
   <si>
-    <t>2026-10-07T15:55:19.711Z</t>
+    <t>2026-10-07T16:28:42.503Z</t>
   </si>
   <si>
     <t>Undergraduate | U-M LSA U-M College of LSA</t>
@@ -338,7 +338,7 @@
     <t>psych/prospective-students/undergraduate</t>
   </si>
   <si>
-    <t>2026-10-07T15:51:13.626Z</t>
+    <t>2026-10-07T15:55:44.221Z</t>
   </si>
   <si>
     <t>Undergraduate | U-M LSA Department of Psychology</t>

</xml_diff>